<commit_message>
42. Trapping Rain Water
</commit_message>
<xml_diff>
--- a/DSA_Interview_Prep_v2.xlsx
+++ b/DSA_Interview_Prep_v2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DSA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBF59E06-AC7B-40E3-B405-B80E17D8EF30}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E99864B5-E526-45FE-AC19-2A51C7F8EF87}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15345" windowHeight="4380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7425" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DSA Questions" sheetId="1" r:id="rId1"/>
@@ -3366,7 +3366,7 @@
       <c r="A6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="45" t="s">
         <v>12</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -3436,7 +3436,7 @@
       <c r="A8" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="45" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="2" t="s">

</xml_diff>

<commit_message>
Subarray Product Less Than K
</commit_message>
<xml_diff>
--- a/DSA_Interview_Prep_v2.xlsx
+++ b/DSA_Interview_Prep_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DSA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E99864B5-E526-45FE-AC19-2A51C7F8EF87}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F87009C2-DB24-4E48-B9F7-CB14C6249B34}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7425" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2583,7 +2583,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2623,6 +2623,14 @@
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="17">
@@ -2733,10 +2741,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2869,8 +2878,12 @@
     <xf numFmtId="0" fontId="2" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -3519,7 +3532,7 @@
       <c r="A11" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="45" t="s">
         <v>46</v>
       </c>
       <c r="C11" s="2" t="s">
@@ -3531,7 +3544,7 @@
       <c r="E11" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F11" s="46" t="s">
         <v>48</v>
       </c>
       <c r="G11" s="2">
@@ -13479,6 +13492,9 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:K1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <hyperlinks>
+    <hyperlink ref="F11" r:id="rId1" xr:uid="{205D3FE5-2D95-4EFF-AA1E-1D14716F867D}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>